<commit_message>
Sorting files before comparing
</commit_message>
<xml_diff>
--- a/Product_16/differences_only.xlsx
+++ b/Product_16/differences_only.xlsx
@@ -1284,10 +1284,8 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>135</t>
-        </is>
+      <c r="G8" s="2" t="n">
+        <v>-1000</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>

</xml_diff>